<commit_message>
Fixed parsing of spreadsheet rows with italics etc
</commit_message>
<xml_diff>
--- a/spec/fixtures/sample_import_assessments.xlsx
+++ b/spec/fixtures/sample_import_assessments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dms3/Desktop/exercises/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B6144A5A-C7DF-4B4A-9FFE-DFE19528653F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{607C9440-27A2-9448-B82D-2BC054787E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="780" windowWidth="28040" windowHeight="17240" xr2:uid="{58324B81-82B1-E942-ADDD-32BBC418C366}"/>
+    <workbookView xWindow="1100" yWindow="680" windowWidth="28040" windowHeight="17240" xr2:uid="{58324B81-82B1-E942-ADDD-32BBC418C366}"/>
   </bookViews>
   <sheets>
     <sheet name="Evaluation World History Vol 1 " sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="53" uniqueCount="48">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="57" uniqueCount="51">
   <si>
     <t>Section</t>
   </si>
@@ -169,13 +169,55 @@
   </si>
   <si>
     <t>e9779614-2fca-43cb-ae53-4af6d20e00ea</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A question with </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>italics</t>
+    </r>
+  </si>
+  <si>
+    <t>It works</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It does </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> work</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -310,6 +352,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -492,7 +547,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <start/>
       <end/>
@@ -607,6 +662,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <start style="thin">
+        <color rgb="FF000000"/>
+      </start>
+      <end style="thin">
+        <color rgb="FF000000"/>
+      </end>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -652,8 +722,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1009,7 +1080,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64FBECA4-7BDF-7B4A-92B0-936D12019FFC}">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -1214,6 +1285,20 @@
         <v>42</v>
       </c>
     </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="H6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M6" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>